<commit_message>
Updated Readme and Project Files
</commit_message>
<xml_diff>
--- a/ProjectFiles/Process Maps.xlsx
+++ b/ProjectFiles/Process Maps.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Birmingham\Dissertation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Birmingham\Dissertation\AcademicHelper\ProjectFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="114">
   <si>
     <t>Current Action / State</t>
   </si>
@@ -41,9 +41,6 @@
     <t>If NO (Next Action)</t>
   </si>
   <si>
-    <t>Source Code Target</t>
-  </si>
-  <si>
     <t>Visitor submits Registration Form</t>
   </si>
   <si>
@@ -53,15 +50,9 @@
     <t>Reject Form &amp; Show Validation Error</t>
   </si>
   <si>
-    <t>app/forms.py</t>
-  </si>
-  <si>
     <t>Form input validation passes</t>
   </si>
   <si>
-    <t>app/routes.py</t>
-  </si>
-  <si>
     <t>Auto-approval trigger active</t>
   </si>
   <si>
@@ -125,9 +116,6 @@
     <t>Storage Destination</t>
   </si>
   <si>
-    <t>Backend Logic</t>
-  </si>
-  <si>
     <t>Upload Gateway</t>
   </si>
   <si>
@@ -158,9 +146,6 @@
     <t>Application Runtime Memory</t>
   </si>
   <si>
-    <t>app/models.py</t>
-  </si>
-  <si>
     <t>Noise Filtering Loop</t>
   </si>
   <si>
@@ -198,9 +183,6 @@
   </si>
   <si>
     <t>Clearance Filtering Matrix</t>
-  </si>
-  <si>
-    <t>Core Framework</t>
   </si>
   <si>
     <t>RAG-01</t>
@@ -266,9 +248,6 @@
     <t>RAG-03</t>
   </si>
   <si>
-    <t>Vector Similarity Query</t>
-  </si>
-  <si>
     <t>Match question coordinates to database indices</t>
   </si>
   <si>
@@ -278,9 +257,6 @@
     <t>Context Splicing</t>
   </si>
   <si>
-    <t>Isolate top 3 nearest matching paragraphs</t>
-  </si>
-  <si>
     <t>Extract text bodies + source + page keys</t>
   </si>
   <si>
@@ -317,9 +293,6 @@
     <t>Data Operation Task</t>
   </si>
   <si>
-    <t>Target Path</t>
-  </si>
-  <si>
     <t>DEL-01</t>
   </si>
   <si>
@@ -344,9 +317,6 @@
     <t>Trigger async JSON fetch block containing target filename</t>
   </si>
   <si>
-    <t>Frontend UI View</t>
-  </si>
-  <si>
     <t>DEL-03</t>
   </si>
   <si>
@@ -374,9 +344,6 @@
     <t>Client-side JavaScript</t>
   </si>
   <si>
-    <t>UI Frontend DOM</t>
-  </si>
-  <si>
     <t>Document Deletion &amp; Disk Purge Process</t>
   </si>
   <si>
@@ -416,32 +383,32 @@
     <t>Verify path in the folder and erase physical file</t>
   </si>
   <si>
-    <t>chroma_db/ index</t>
-  </si>
-  <si>
     <t>Remove all vector segments where where filename matches the selection</t>
   </si>
   <si>
-    <t>../uploads/ directory</t>
-  </si>
-  <si>
     <t>Evict target table row from Document Object Model via .remove() wrapper</t>
   </si>
   <si>
-    <t>Tracks log to SQLite chat_message</t>
-  </si>
-  <si>
     <t>Filter results strictly by allowed tier list</t>
   </si>
   <si>
     <t>Inject answer and citation keys into view</t>
+  </si>
+  <si>
+    <t>Isolate top 4 nearest matching paragraphs</t>
+  </si>
+  <si>
+    <t>Hybrid Search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracks log to SQLite </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -461,12 +428,6 @@
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Google Sans Text"/>
       <family val="2"/>
     </font>
     <font>
@@ -564,7 +525,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -572,11 +533,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
@@ -584,6 +542,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -602,18 +563,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -896,26 +845,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.5546875" customWidth="1"/>
     <col min="2" max="2" width="26.77734375" customWidth="1"/>
     <col min="3" max="3" width="22.77734375" customWidth="1"/>
     <col min="4" max="4" width="25.21875" customWidth="1"/>
     <col min="5" max="5" width="22.21875" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6">
-      <c r="A1" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15" thickBot="1"/>
-    <row r="3" spans="1:6" ht="28.2" thickBot="1">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>0</v>
@@ -929,108 +877,90 @@
       <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="28.2" thickBot="1">
+    </row>
+    <row r="4" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="28.2" thickBot="1">
+    </row>
+    <row r="5" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="28.2" thickBot="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.2" thickBot="1">
+    <row r="7" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="28.2" thickBot="1">
+    <row r="8" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1041,156 +971,135 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="14.4"/>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15" thickBot="1"/>
-    <row r="3" spans="1:6" ht="15" thickBot="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="28.2" thickBot="1">
-      <c r="A4" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="5" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E5" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="28.2" thickBot="1">
-      <c r="A5" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="2" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="28.2" thickBot="1">
-      <c r="A6" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E6" s="2" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="C8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="28.2" thickBot="1">
-      <c r="A7" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" s="2" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="28.2" thickBot="1">
-      <c r="A8" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="28.2" thickBot="1">
-      <c r="A9" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1201,178 +1110,151 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" customWidth="1"/>
     <col min="2" max="3" width="21.88671875" customWidth="1"/>
     <col min="4" max="4" width="41.88671875" customWidth="1"/>
-    <col min="5" max="5" width="21.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1"/>
-    <row r="3" spans="1:5" ht="15" thickBot="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D4" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="B5" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="C5" s="12" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A4" s="1" t="s">
+      <c r="D5" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="16"/>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
-      <c r="D7" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E7" s="16"/>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="D7" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="10"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="16"/>
-    </row>
-    <row r="9" spans="1:5" ht="15" thickBot="1">
+      <c r="D8" s="8"/>
+    </row>
+    <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11"/>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="17"/>
-    </row>
-    <row r="10" spans="1:5" ht="42" thickBot="1">
-      <c r="A10" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A11" s="1" t="s">
+    </row>
+    <row r="13" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="42" thickBot="1">
-      <c r="A12" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="42" thickBot="1">
-      <c r="A13" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>10</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="B5:B9"/>
     <mergeCell ref="C5:C9"/>
-    <mergeCell ref="E5:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1380,119 +1262,101 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="5" width="29.44140625" customWidth="1"/>
+    <col min="2" max="4" width="29.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6">
-      <c r="A1" s="5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1"/>
-    <row r="3" spans="1:5" ht="15" thickBot="1">
+    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E3" s="1" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A4" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="42" thickBot="1">
-      <c r="A5" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="42" thickBot="1">
-      <c r="A6" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="28.2" thickBot="1">
-      <c r="A7" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="42" thickBot="1">
-      <c r="A8" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>